<commit_message>
Add 13 reference PDFs, updated litteratursporing and Gantt charts
- 13 nye artikler lagt til i 003 references (METRIC-familien, spare parts, PPE)
- Litteratursporing_LOG650_G20.xlsx oppdatert
- Gantt v2 og v3 lagt til i 012 fase 2 - plan
- .pdf (navnløs fil) holdt utenfor — avklares separat

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/003 references/Litteratursporing_LOG650_G20.xlsx
+++ b/003 references/Litteratursporing_LOG650_G20.xlsx
@@ -5,26 +5,26 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\runeg\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/be25ac4905db4876/Documents/Skole utdanning/Logistikk studie/LOG650 LOGISTIKK OG KI/G20-rune-individuell/003 references/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1BAFD95-4696-41C1-ADFA-4E558B05AFA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="47" documentId="13_ncr:1_{D1BAFD95-4696-41C1-ADFA-4E558B05AFA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4CCB9D04-72B8-49D7-95AF-64676DD6A6C9}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15" yWindow="525" windowWidth="21585" windowHeight="12255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Litteratursporing" sheetId="1" r:id="rId1"/>
     <sheet name="Forklaring" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Litteratursporing!$A$1:$M$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Litteratursporing!$A$1:$M$23</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="150">
   <si>
     <t>Pri</t>
   </si>
@@ -110,9 +110,6 @@
     <t>Bok</t>
   </si>
   <si>
-    <t>10.1007/b109856</t>
-  </si>
-  <si>
     <t>SpringerLink (HiMolde)</t>
   </si>
   <si>
@@ -260,9 +257,6 @@
     <t>The (S-1,S) inventory policy under compound Poisson demand</t>
   </si>
   <si>
-    <t>10.1287/mnsc.9.3.391</t>
-  </si>
-  <si>
     <t>Verifiser DOI</t>
   </si>
   <si>
@@ -290,9 +284,6 @@
     <t>Expediting in two-echelon spare parts inventory systems</t>
   </si>
   <si>
-    <t>10.1287/msom.2020.0888</t>
-  </si>
-  <si>
     <t>Jernbane-case</t>
   </si>
   <si>
@@ -305,9 +296,6 @@
     <t>Spare parts inventory control under system availability constraints</t>
   </si>
   <si>
-    <t>10.1007/978-1-4615-4195-8</t>
-  </si>
-  <si>
     <t>Srivathsan &amp; Viswanathan 2017</t>
   </si>
   <si>
@@ -353,9 +341,6 @@
     <t>The effect of personal protective equipment on firefighter occupational performance</t>
   </si>
   <si>
-    <t>10.1080/15459624.2019.1692684</t>
-  </si>
-  <si>
     <t>PubMed</t>
   </si>
   <si>
@@ -483,6 +468,12 @@
   </si>
   <si>
     <t>følger anbefalt rekkefølge fra litteraturlisten</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/springer_10.1007-b109856</t>
+  </si>
+  <si>
+    <t>NEI</t>
   </si>
 </sst>
 </file>
@@ -649,6 +640,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1023,8 +1018,12 @@
       <c r="I2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
+      <c r="J2" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>34</v>
+      </c>
       <c r="L2" s="3"/>
       <c r="M2" s="2"/>
     </row>
@@ -1056,8 +1055,12 @@
       <c r="I3" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
+      <c r="J3" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>34</v>
+      </c>
       <c r="L3" s="5"/>
       <c r="M3" s="4"/>
     </row>
@@ -1084,13 +1087,17 @@
         <v>27</v>
       </c>
       <c r="H4" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I4" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
+      <c r="J4" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>34</v>
+      </c>
       <c r="L4" s="3"/>
       <c r="M4" s="2"/>
     </row>
@@ -1102,13 +1109,13 @@
         <v>13</v>
       </c>
       <c r="C5" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>31</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>32</v>
       </c>
       <c r="F5" s="4">
         <v>2015</v>
@@ -1117,20 +1124,20 @@
         <v>27</v>
       </c>
       <c r="H5" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="I5" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="I5" s="4" t="s">
-        <v>34</v>
-      </c>
       <c r="J5" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="L5" s="5"/>
       <c r="M5" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.45">
@@ -1141,13 +1148,13 @@
         <v>13</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="F6" s="2">
         <v>1997</v>
@@ -1156,13 +1163,17 @@
         <v>17</v>
       </c>
       <c r="H6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="I6" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="I6" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
+      <c r="J6" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>34</v>
+      </c>
       <c r="L6" s="3"/>
       <c r="M6" s="2"/>
     </row>
@@ -1174,13 +1185,13 @@
         <v>13</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>43</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>44</v>
       </c>
       <c r="F7" s="4">
         <v>2014</v>
@@ -1189,13 +1200,17 @@
         <v>17</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
+        <v>40</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>34</v>
+      </c>
       <c r="L7" s="5"/>
       <c r="M7" s="4"/>
     </row>
@@ -1204,16 +1219,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>46</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>47</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>15</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F8" s="6">
         <v>1986</v>
@@ -1222,10 +1237,10 @@
         <v>17</v>
       </c>
       <c r="H8" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="I8" s="6" t="s">
         <v>49</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>50</v>
       </c>
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
@@ -1237,16 +1252,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C9" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="E9" s="8" t="s">
         <v>52</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>53</v>
       </c>
       <c r="F9" s="8">
         <v>1973</v>
@@ -1255,16 +1270,20 @@
         <v>17</v>
       </c>
       <c r="H9" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="I9" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="I9" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
+      <c r="J9" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="K9" s="9" t="s">
+        <v>34</v>
+      </c>
       <c r="L9" s="9"/>
       <c r="M9" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.45">
@@ -1272,31 +1291,35 @@
         <v>9</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C10" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D10" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="E10" s="6" t="s">
         <v>58</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>59</v>
       </c>
       <c r="F10" s="6">
         <v>1982</v>
       </c>
       <c r="G10" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="H10" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="H10" s="6" t="s">
+      <c r="I10" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="I10" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="J10" s="7"/>
-      <c r="K10" s="7"/>
+      <c r="J10" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>34</v>
+      </c>
       <c r="L10" s="7"/>
       <c r="M10" s="6"/>
     </row>
@@ -1305,16 +1328,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C11" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="D11" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="E11" s="8" t="s">
         <v>64</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>65</v>
       </c>
       <c r="F11" s="8">
         <v>2021</v>
@@ -1323,13 +1346,17 @@
         <v>17</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="J11" s="9"/>
-      <c r="K11" s="9"/>
+        <v>40</v>
+      </c>
+      <c r="J11" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="K11" s="9" t="s">
+        <v>34</v>
+      </c>
       <c r="L11" s="9"/>
       <c r="M11" s="8"/>
     </row>
@@ -1338,16 +1365,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C12" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="D12" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="E12" s="6" t="s">
         <v>68</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>69</v>
       </c>
       <c r="F12" s="6">
         <v>2019</v>
@@ -1356,13 +1383,17 @@
         <v>17</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="J12" s="7"/>
-      <c r="K12" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J12" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="K12" s="7" t="s">
+        <v>34</v>
+      </c>
       <c r="L12" s="7"/>
       <c r="M12" s="6"/>
     </row>
@@ -1371,16 +1402,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C13" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="D13" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="E13" s="8" t="s">
         <v>72</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>73</v>
       </c>
       <c r="F13" s="8">
         <v>2011</v>
@@ -1389,13 +1420,17 @@
         <v>17</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="J13" s="9"/>
-      <c r="K13" s="9"/>
+        <v>40</v>
+      </c>
+      <c r="J13" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="K13" s="9" t="s">
+        <v>34</v>
+      </c>
       <c r="L13" s="9"/>
       <c r="M13" s="8"/>
     </row>
@@ -1404,16 +1439,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C14" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="D14" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="E14" s="6" t="s">
         <v>76</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>77</v>
       </c>
       <c r="F14" s="6">
         <v>1963</v>
@@ -1421,17 +1456,15 @@
       <c r="G14" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="H14" s="6" t="s">
-        <v>78</v>
-      </c>
+      <c r="H14" s="6"/>
       <c r="I14" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J14" s="7"/>
       <c r="K14" s="7"/>
       <c r="L14" s="7"/>
       <c r="M14" s="6" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.45">
@@ -1439,16 +1472,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C15" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="E15" s="8" t="s">
         <v>80</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>82</v>
       </c>
       <c r="F15" s="8">
         <v>1987</v>
@@ -1457,13 +1490,17 @@
         <v>17</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="J15" s="9"/>
-      <c r="K15" s="9"/>
+        <v>82</v>
+      </c>
+      <c r="J15" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="K15" s="9" t="s">
+        <v>34</v>
+      </c>
       <c r="L15" s="9"/>
       <c r="M15" s="8"/>
     </row>
@@ -1472,16 +1509,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C16" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="E16" s="6" t="s">
         <v>85</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>87</v>
       </c>
       <c r="F16" s="6">
         <v>2021</v>
@@ -1489,17 +1526,15 @@
       <c r="G16" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="H16" s="6" t="s">
-        <v>88</v>
-      </c>
+      <c r="H16" s="6"/>
       <c r="I16" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J16" s="7"/>
       <c r="K16" s="7"/>
       <c r="L16" s="7"/>
       <c r="M16" s="6" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.45">
@@ -1507,16 +1542,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="F17" s="8">
         <v>2015</v>
@@ -1524,17 +1559,15 @@
       <c r="G17" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="H17" s="8" t="s">
-        <v>93</v>
-      </c>
+      <c r="H17" s="8"/>
       <c r="I17" s="8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J17" s="9"/>
       <c r="K17" s="9"/>
       <c r="L17" s="9"/>
       <c r="M17" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.45">
@@ -1542,16 +1575,16 @@
         <v>17</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="F18" s="6">
         <v>2017</v>
@@ -1560,16 +1593,20 @@
         <v>17</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="J18" s="7"/>
-      <c r="K18" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>34</v>
+      </c>
       <c r="L18" s="7"/>
       <c r="M18" s="6" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.45">
@@ -1577,16 +1614,16 @@
         <v>18</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="F19" s="8">
         <v>2019</v>
@@ -1595,13 +1632,17 @@
         <v>17</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="J19" s="9"/>
-      <c r="K19" s="9"/>
+        <v>40</v>
+      </c>
+      <c r="J19" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="K19" s="9" t="s">
+        <v>34</v>
+      </c>
       <c r="L19" s="9"/>
       <c r="M19" s="8"/>
     </row>
@@ -1610,16 +1651,16 @@
         <v>19</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="F20" s="6">
         <v>2018</v>
@@ -1628,13 +1669,17 @@
         <v>17</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="J20" s="7"/>
-      <c r="K20" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J20" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="K20" s="7" t="s">
+        <v>34</v>
+      </c>
       <c r="L20" s="7"/>
       <c r="M20" s="6"/>
     </row>
@@ -1643,16 +1688,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="F21" s="8">
         <v>2020</v>
@@ -1660,17 +1705,19 @@
       <c r="G21" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H21" s="8" t="s">
-        <v>109</v>
-      </c>
+      <c r="H21" s="8"/>
       <c r="I21" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="J21" s="9"/>
-      <c r="K21" s="9"/>
+        <v>105</v>
+      </c>
+      <c r="J21" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="K21" s="9" t="s">
+        <v>34</v>
+      </c>
       <c r="L21" s="9"/>
       <c r="M21" s="8" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.45">
@@ -1678,31 +1725,35 @@
         <v>21</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="F22" s="10">
         <v>2022</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="H22" s="10" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="J22" s="11"/>
-      <c r="K22" s="11"/>
+        <v>113</v>
+      </c>
+      <c r="J22" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="K22" s="11" t="s">
+        <v>34</v>
+      </c>
       <c r="L22" s="11"/>
       <c r="M22" s="10"/>
     </row>
@@ -1711,38 +1762,42 @@
         <v>22</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="E23" s="12" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="F23" s="12">
         <v>2022</v>
       </c>
       <c r="G23" s="12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H23" s="12" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="I23" s="12" t="s">
-        <v>122</v>
-      </c>
-      <c r="J23" s="13"/>
-      <c r="K23" s="13"/>
+        <v>117</v>
+      </c>
+      <c r="J23" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="K23" s="13" t="s">
+        <v>34</v>
+      </c>
       <c r="L23" s="13"/>
       <c r="M23" s="12" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:M23" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1758,10 +1813,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A1" s="14" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.45">
@@ -1769,7 +1824,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="25.5" x14ac:dyDescent="0.45">
@@ -1777,7 +1832,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.45">
@@ -1785,7 +1840,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.45">
@@ -1793,7 +1848,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.45">
@@ -1801,7 +1856,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.45">
@@ -1809,7 +1864,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.45">
@@ -1817,7 +1872,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.45">
@@ -1825,7 +1880,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.45">
@@ -1833,7 +1888,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.45">
@@ -1841,7 +1896,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.45">
@@ -1849,7 +1904,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.45">
@@ -1857,7 +1912,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.45">
@@ -1865,7 +1920,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.45">
@@ -1874,32 +1929,32 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A16" s="14" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="B16" s="15"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A17" s="15" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A18" s="15" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A19" s="15" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.45">
@@ -1908,32 +1963,32 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A21" s="14" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B21" s="15"/>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A22" s="15" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A23" s="15" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A24" s="15" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>